<commit_message>
row count columns now BIGINT
</commit_message>
<xml_diff>
--- a/apcd_export_import/apcd_etl_log.xlsx
+++ b/apcd_export_import/apcd_etl_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kc1-my.sharepoint.com/personal/jwhitehurst_kingcounty_gov/Documents/GitHub/claims_data/apcd_export_import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_F25DC773A252ABDACC10489BD19F75405ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BB55FCD-76B0-414A-85B3-390D022D33DF}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_F25DC773A252ABDACC10489BD19F75405ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D962F5B5-1B91-4B8D-8DF0-75C1CD0240F9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="19545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -72,9 +72,6 @@
     <t>rows_file</t>
   </si>
   <si>
-    <t>INTEGER</t>
-  </si>
-  <si>
     <t>rows_loaded</t>
   </si>
   <si>
@@ -109,6 +106,9 @@
   </si>
   <si>
     <t>column_position</t>
+  </si>
+  <si>
+    <t>BIGINT</t>
   </si>
 </sst>
 </file>
@@ -439,19 +439,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" t="s">
         <v>26</v>
-      </c>
-      <c r="E1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -584,7 +584,7 @@
         <v>14</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E9">
         <v>8</v>
@@ -598,10 +598,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -615,10 +615,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -632,10 +632,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E12">
         <v>11</v>
@@ -649,10 +649,10 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E13">
         <v>12</v>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14">
         <v>13</v>
@@ -683,10 +683,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E15">
         <v>14</v>

</xml_diff>